<commit_message>
Add finished judgements with introductory beginning
</commit_message>
<xml_diff>
--- a/debug/judgements_intro/excel_overviews/gpt-4.1_vs_Llama-2-7b-chat-hf/Llama-3.3-70B-Instruct/aae/total_votes_file.xlsx
+++ b/debug/judgements_intro/excel_overviews/gpt-4.1_vs_Llama-2-7b-chat-hf/Llama-3.3-70B-Instruct/aae/total_votes_file.xlsx
@@ -430,13 +430,13 @@
         <v>7</v>
       </c>
       <c r="C2">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D2">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -450,13 +450,13 @@
         <v>8</v>
       </c>
       <c r="C3">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D3">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
         <v>0</v>

</xml_diff>